<commit_message>
docs: replace bom due to recalculation
</commit_message>
<xml_diff>
--- a/production/breadboard-power-qcpd-bom.xlsx
+++ b/production/breadboard-power-qcpd-bom.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10802"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\ПРОЧЕЕ\Колледж\5 курс\Дипломы\.Работы\В РАБОТЕ\...МОЙ\Диплом\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aiurat/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A86E02-EB08-41D1-A6A0-8BBA44DF2089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA335C53-61CF-6141-AB5F-21E45BADC399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8145" yWindow="900" windowWidth="20700" windowHeight="13440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="89">
   <si>
     <t>Элементы</t>
   </si>
@@ -48,21 +48,12 @@
     <t>Номиналы</t>
   </si>
   <si>
-    <t>0,22 Ом</t>
-  </si>
-  <si>
     <t>1 кОм</t>
   </si>
   <si>
     <t>10 кОм</t>
   </si>
   <si>
-    <t>Наличие</t>
-  </si>
-  <si>
-    <t>2,2 нФ</t>
-  </si>
-  <si>
     <t>1 мкФ</t>
   </si>
   <si>
@@ -222,9 +213,6 @@
     <t>R0603</t>
   </si>
   <si>
-    <t>https://www.chipdip.ru/product0/8007033652</t>
-  </si>
-  <si>
     <t>https://www.chipdip.ru/product0/8014349442</t>
   </si>
   <si>
@@ -258,9 +246,6 @@
     <t>220 мкГн</t>
   </si>
   <si>
-    <t>https://www.chipdip.ru/product0/8004352023</t>
-  </si>
-  <si>
     <t>https://www.chipdip.ru/product0/8008634629</t>
   </si>
   <si>
@@ -270,36 +255,18 @@
     <t>MS-22D16G2-B COPY</t>
   </si>
   <si>
-    <t>7+9</t>
-  </si>
-  <si>
-    <t>6(+47)</t>
-  </si>
-  <si>
-    <t>910 Ом</t>
-  </si>
-  <si>
-    <t>R1, R2, R5, R6, R7</t>
-  </si>
-  <si>
     <t>R8, R9</t>
   </si>
   <si>
     <t>https://www.chipdip.ru/product/0.1w-0603-10-kom-5</t>
   </si>
   <si>
-    <t>https://www.chipdip.ru/product/0.1w-0603-910-om-5</t>
-  </si>
-  <si>
     <t>https://www.chipdip.ru/product/0.1w-0603-1-kom-5</t>
   </si>
   <si>
     <t>100 пФ</t>
   </si>
   <si>
-    <t>5(+4)</t>
-  </si>
-  <si>
     <t>R2512</t>
   </si>
   <si>
@@ -309,15 +276,9 @@
     <t>https://www.chipdip.ru/product/b82464g4224m</t>
   </si>
   <si>
-    <t>ЗАМЕНА ПО РАСЧЁТАМ</t>
-  </si>
-  <si>
     <t>0,3 Ом</t>
   </si>
   <si>
-    <t>всего</t>
-  </si>
-  <si>
     <t>R1</t>
   </si>
   <si>
@@ -337,6 +298,9 @@
   </si>
   <si>
     <t>https://www.chipdip.ru/product/grm1885c1h101j</t>
+  </si>
+  <si>
+    <t>R2, R5, R6, R7</t>
   </si>
 </sst>
 </file>
@@ -387,11 +351,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -675,30 +642,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="56.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="48.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -707,63 +674,54 @@
         <v>2</v>
       </c>
       <c r="G1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B2" t="s">
         <v>81</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>6</v>
+        <v>82</v>
       </c>
       <c r="F2" s="2">
+        <v>1</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="I2" s="2"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="2">
-        <v>31</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2">
         <v>4</v>
       </c>
-      <c r="F3" s="2">
-        <v>1</v>
-      </c>
-      <c r="G3" s="2">
-        <v>9</v>
-      </c>
-      <c r="H3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>74</v>
       </c>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="C4" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>80</v>
@@ -771,472 +729,393 @@
       <c r="F4" s="2">
         <v>1</v>
       </c>
-      <c r="G4" s="2">
-        <v>16</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>84</v>
-      </c>
+      <c r="G4" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="H4" s="1"/>
       <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>82</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>5</v>
+        <v>83</v>
       </c>
       <c r="F5" s="2">
+        <v>1</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" s="2">
         <v>2</v>
       </c>
-      <c r="G5" s="2">
-        <v>14</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="I5" s="2"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="2">
-        <v>1</v>
-      </c>
-      <c r="G6" s="2">
-        <v>99</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>62</v>
+      <c r="G6" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>60</v>
+      </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C7" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>9</v>
+        <v>27</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>76</v>
       </c>
       <c r="F7" s="2">
         <v>1</v>
       </c>
-      <c r="G7" s="2">
-        <v>9</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>23</v>
+      <c r="G7" s="1" t="s">
+        <v>87</v>
       </c>
       <c r="I7" s="2"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="F8" s="2">
         <v>1</v>
       </c>
-      <c r="G8" s="2">
-        <v>6</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>25</v>
+      <c r="G8" s="1" t="s">
+        <v>20</v>
       </c>
       <c r="I8" s="2"/>
       <c r="L8" s="2"/>
       <c r="O8" s="1"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F9" s="2">
-        <v>2</v>
-      </c>
-      <c r="G9" s="2">
-        <v>12</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>24</v>
+        <v>1</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="I9" s="2"/>
       <c r="L9" s="2"/>
       <c r="O9" s="1"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>65</v>
-      </c>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C10" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E10" s="2"/>
+        <v>32</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>7</v>
+      </c>
       <c r="F10" s="2">
-        <v>1</v>
-      </c>
-      <c r="G10" s="2">
-        <v>30</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>63</v>
+        <v>2</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="I10" s="2"/>
       <c r="L10" s="2"/>
       <c r="O10" s="1"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="D11" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="2">
         <v>1</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>21</v>
+      <c r="G11" s="1" t="s">
+        <v>59</v>
       </c>
       <c r="I11" s="2"/>
       <c r="L11" s="2"/>
       <c r="O11" s="1"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>15</v>
-      </c>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" t="s">
         <v>39</v>
       </c>
-      <c r="C12" t="s">
-        <v>40</v>
-      </c>
       <c r="D12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" s="2">
         <v>1</v>
       </c>
-      <c r="G12" s="2">
-        <v>6</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>20</v>
+      <c r="G12" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="I12" s="2"/>
       <c r="L12" s="2"/>
       <c r="O12" s="1"/>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="D13" t="s">
-        <v>43</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>73</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="E13" s="2"/>
       <c r="F13" s="2">
         <v>1</v>
       </c>
-      <c r="G13" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>90</v>
+      <c r="G13" s="1" t="s">
+        <v>17</v>
       </c>
       <c r="I13" s="2"/>
       <c r="O13" s="1"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>67</v>
       </c>
       <c r="B14" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C14" t="s">
-        <v>76</v>
+        <v>42</v>
       </c>
       <c r="D14" t="s">
-        <v>77</v>
-      </c>
-      <c r="E14" s="2"/>
+        <v>40</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>69</v>
+      </c>
       <c r="F14" s="2">
-        <v>2</v>
-      </c>
-      <c r="G14" s="2">
-        <v>12</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>75</v>
+        <v>1</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>79</v>
       </c>
       <c r="I14" s="2"/>
       <c r="O14" s="1"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>8</v>
+      </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>71</v>
       </c>
       <c r="D15" t="s">
-        <v>13</v>
+        <v>72</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2">
-        <v>1</v>
-      </c>
-      <c r="G15" s="2">
-        <v>6</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>19</v>
+        <v>2</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>70</v>
       </c>
       <c r="I15" s="2"/>
       <c r="O15" s="1"/>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>67</v>
-      </c>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="D16" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2">
         <v>1</v>
       </c>
-      <c r="G16" s="2">
-        <v>6</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>70</v>
+      <c r="G16" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="I16" s="2"/>
       <c r="O16" s="1"/>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B17" t="s">
-        <v>89</v>
+        <v>48</v>
       </c>
       <c r="C17" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D17" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" s="2">
         <v>1</v>
       </c>
-      <c r="G17" s="2">
-        <v>6</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>69</v>
+      <c r="G17" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="I17" s="2"/>
       <c r="O17" s="1"/>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>64</v>
       </c>
       <c r="B18" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="C18" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D18" t="s">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2">
         <v>1</v>
       </c>
-      <c r="G18" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>22</v>
+      <c r="G18" s="1" t="s">
+        <v>65</v>
       </c>
       <c r="I18" s="2"/>
       <c r="O18" s="1"/>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>14</v>
+      </c>
       <c r="B19" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C19" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D19" t="s">
-        <v>57</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="E19" s="2"/>
       <c r="F19" s="2">
-        <v>2</v>
-      </c>
-      <c r="G19" s="2">
-        <v>12</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>66</v>
+        <v>1</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="I19" s="2"/>
       <c r="O19" s="1"/>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="E20" s="2" t="s">
-        <v>93</v>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" t="s">
+        <v>54</v>
       </c>
       <c r="F20" s="2">
-        <f>SUM(F2:F19)</f>
-        <v>26</v>
-      </c>
-      <c r="G20" s="2"/>
-      <c r="H20" s="1"/>
+        <v>2</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>62</v>
+      </c>
       <c r="O20" s="1"/>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>91</v>
-      </c>
-      <c r="B21" t="s">
-        <v>29</v>
-      </c>
-      <c r="C21" t="s">
-        <v>86</v>
-      </c>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="G21" s="2"/>
-      <c r="H21" s="1" t="s">
-        <v>100</v>
-      </c>
+      <c r="H21" s="1"/>
       <c r="O21" s="1"/>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
-        <v>94</v>
-      </c>
-      <c r="C22" t="s">
-        <v>95</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>97</v>
-      </c>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="H22" s="1"/>
       <c r="O22" s="1"/>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B23" t="s">
-        <v>46</v>
-      </c>
-      <c r="C23" t="s">
-        <v>92</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>98</v>
-      </c>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="H23" s="1"/>
       <c r="O23" s="1"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B24" t="s">
-        <v>28</v>
-      </c>
-      <c r="C24" t="s">
-        <v>96</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>99</v>
-      </c>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="H24" s="1"/>
       <c r="O24" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="H6" r:id="rId1" xr:uid="{8B07012F-18B8-4174-B921-549BFF0E5AA3}"/>
-    <hyperlink ref="H7" r:id="rId2" xr:uid="{F7C3E5D0-B415-45F0-9F31-0765D8F4D390}"/>
-    <hyperlink ref="H8" r:id="rId3" xr:uid="{BDCFA3F8-EFDF-4974-8764-78A26FD8F1D8}"/>
-    <hyperlink ref="H9" r:id="rId4" xr:uid="{809570E2-141A-47CE-A1DA-A6FDC2A9C184}"/>
-    <hyperlink ref="H10" r:id="rId5" xr:uid="{02FCAB2F-1BA1-4CD3-9EE1-E9AE98B12B6E}"/>
-    <hyperlink ref="H12" r:id="rId6" xr:uid="{E58FF732-51F3-47A7-AA80-872B35B79C91}"/>
-    <hyperlink ref="H18" r:id="rId7" xr:uid="{4359FD89-2BDD-4EE2-B299-F3F5D61BC9C0}"/>
-    <hyperlink ref="H19" r:id="rId8" xr:uid="{5BCC7B57-F23D-435F-8DFA-8ABA07EA63A7}"/>
-    <hyperlink ref="H17" r:id="rId9" xr:uid="{20206CD3-5586-4298-A261-F94B8885C31F}"/>
-    <hyperlink ref="H16" r:id="rId10" xr:uid="{D2ECFF2A-F76C-4F5F-A01D-930545D9BBB1}"/>
-    <hyperlink ref="H13" r:id="rId11" xr:uid="{3C42E7A9-B52C-495B-8DD9-0EACBB538694}"/>
-    <hyperlink ref="H15" r:id="rId12" xr:uid="{F35E4B90-88FC-4D0E-BB72-F7D7824A9719}"/>
-    <hyperlink ref="H3" r:id="rId13" xr:uid="{5D3E44A2-0496-4117-B6F4-033D5C9A5E35}"/>
-    <hyperlink ref="H14" r:id="rId14" xr:uid="{6BC1E3A6-2DD9-4F68-B517-B3D5A00DE662}"/>
-    <hyperlink ref="H11" r:id="rId15" xr:uid="{6FF73B55-6DCD-4BBD-B61B-7E826135A98A}"/>
-    <hyperlink ref="H5" r:id="rId16" xr:uid="{6EE0AEA4-4F92-4397-8DF0-DBA36561BEBD}"/>
-    <hyperlink ref="H2" r:id="rId17" xr:uid="{76F7F569-627B-4AD7-BB06-05DAC7319877}"/>
-    <hyperlink ref="H4" r:id="rId18" xr:uid="{48CDA878-61BE-45AB-B56F-7653D55E5FEA}"/>
-    <hyperlink ref="H22" r:id="rId19" xr:uid="{4D310CCF-4F3B-4B79-9EDC-9720A9FACE68}"/>
-    <hyperlink ref="H23" r:id="rId20" xr:uid="{5DA96E43-2C6E-41FE-88F2-CC5CA454A29A}"/>
-    <hyperlink ref="H24" r:id="rId21" xr:uid="{DAC700D6-78E6-4CDC-ACE2-FD5C1A6C4D26}"/>
-    <hyperlink ref="H21" r:id="rId22" xr:uid="{20C62ACC-6385-48C6-9F18-7D587B738602}"/>
+    <hyperlink ref="G8" r:id="rId1" xr:uid="{F7C3E5D0-B415-45F0-9F31-0765D8F4D390}"/>
+    <hyperlink ref="G9" r:id="rId2" xr:uid="{BDCFA3F8-EFDF-4974-8764-78A26FD8F1D8}"/>
+    <hyperlink ref="G10" r:id="rId3" xr:uid="{809570E2-141A-47CE-A1DA-A6FDC2A9C184}"/>
+    <hyperlink ref="G11" r:id="rId4" xr:uid="{02FCAB2F-1BA1-4CD3-9EE1-E9AE98B12B6E}"/>
+    <hyperlink ref="G13" r:id="rId5" xr:uid="{E58FF732-51F3-47A7-AA80-872B35B79C91}"/>
+    <hyperlink ref="G19" r:id="rId6" xr:uid="{4359FD89-2BDD-4EE2-B299-F3F5D61BC9C0}"/>
+    <hyperlink ref="G20" r:id="rId7" xr:uid="{5BCC7B57-F23D-435F-8DFA-8ABA07EA63A7}"/>
+    <hyperlink ref="G18" r:id="rId8" xr:uid="{20206CD3-5586-4298-A261-F94B8885C31F}"/>
+    <hyperlink ref="G17" r:id="rId9" xr:uid="{D2ECFF2A-F76C-4F5F-A01D-930545D9BBB1}"/>
+    <hyperlink ref="G14" r:id="rId10" xr:uid="{3C42E7A9-B52C-495B-8DD9-0EACBB538694}"/>
+    <hyperlink ref="G16" r:id="rId11" xr:uid="{F35E4B90-88FC-4D0E-BB72-F7D7824A9719}"/>
+    <hyperlink ref="G15" r:id="rId12" xr:uid="{6BC1E3A6-2DD9-4F68-B517-B3D5A00DE662}"/>
+    <hyperlink ref="G12" r:id="rId13" xr:uid="{6FF73B55-6DCD-4BBD-B61B-7E826135A98A}"/>
+    <hyperlink ref="G6" r:id="rId14" xr:uid="{6EE0AEA4-4F92-4397-8DF0-DBA36561BEBD}"/>
+    <hyperlink ref="G3" r:id="rId15" xr:uid="{76F7F569-627B-4AD7-BB06-05DAC7319877}"/>
+    <hyperlink ref="G7" r:id="rId16" xr:uid="{130FF3EF-2A55-DE48-84D6-021E1982E1EC}"/>
+    <hyperlink ref="G2" r:id="rId17" xr:uid="{55E80D02-0781-1D4D-B902-E33CB9FCA435}"/>
+    <hyperlink ref="G4" r:id="rId18" xr:uid="{BC5DE1AF-45FD-5D47-BD99-DCF732852436}"/>
+    <hyperlink ref="G5" r:id="rId19" xr:uid="{950536A6-995E-4149-8CFC-E2C7CC74FDD9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId23"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId20"/>
 </worksheet>
 </file>
</xml_diff>